<commit_message>
Fix K6 load test report - restore baseline data with 3-sheet format
</commit_message>
<xml_diff>
--- a/test_reports/K6_Load_Test_Report.xlsx
+++ b/test_reports/K6_Load_Test_Report.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -34,23 +34,44 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="001A237E"/>
+      <color rgb="00FFFFFF"/>
       <sz val="11"/>
     </font>
     <font>
+      <color rgb="00E0E0E0"/>
       <sz val="11"/>
     </font>
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="0090CAF9"/>
       <sz val="11"/>
     </font>
     <font>
       <b val="1"/>
-      <color rgb="002E7D32"/>
+      <color rgb="0000E676"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <color rgb="00B0BEC5"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="0069F0AE"/>
+      <sz val="11"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -59,32 +80,47 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="001B1F2A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="006C63FF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00232836"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0037474F"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="003949AB"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00263238"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="001B5E20"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="002E7D32"/>
+        <fgColor rgb="0000695C"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F5F5F5"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="000D47A1"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="001565C0"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="004A148C"/>
+        <fgColor rgb="00E65100"/>
       </patternFill>
     </fill>
   </fills>
@@ -97,66 +133,64 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+      <left style="thin">
+        <color rgb="0037474F"/>
+      </left>
+      <right style="thin">
+        <color rgb="0037474F"/>
+      </right>
+      <top style="thin">
+        <color rgb="0037474F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="0037474F"/>
+      </bottom>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -270,6 +304,116 @@
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
+          <dPt>
+            <idx val="0"/>
+            <spPr>
+              <a:solidFill>
+                <a:srgbClr val="4CAF50"/>
+              </a:solidFill>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </dPt>
+          <dPt>
+            <idx val="1"/>
+            <spPr>
+              <a:solidFill>
+                <a:srgbClr val="2196F3"/>
+              </a:solidFill>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </dPt>
+          <dPt>
+            <idx val="2"/>
+            <spPr>
+              <a:solidFill>
+                <a:srgbClr val="FF9800"/>
+              </a:solidFill>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </dPt>
+          <dPt>
+            <idx val="3"/>
+            <spPr>
+              <a:solidFill>
+                <a:srgbClr val="9C27B0"/>
+              </a:solidFill>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </dPt>
+          <dPt>
+            <idx val="4"/>
+            <spPr>
+              <a:solidFill>
+                <a:srgbClr val="F44336"/>
+              </a:solidFill>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </dPt>
+          <dPt>
+            <idx val="5"/>
+            <spPr>
+              <a:solidFill>
+                <a:srgbClr val="00BCD4"/>
+              </a:solidFill>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </dPt>
+          <dPt>
+            <idx val="6"/>
+            <spPr>
+              <a:solidFill>
+                <a:srgbClr val="795548"/>
+              </a:solidFill>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </dPt>
+          <dPt>
+            <idx val="7"/>
+            <spPr>
+              <a:solidFill>
+                <a:srgbClr val="607D8B"/>
+              </a:solidFill>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </dPt>
+          <dPt>
+            <idx val="8"/>
+            <spPr>
+              <a:solidFill>
+                <a:srgbClr val="E91E63"/>
+              </a:solidFill>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </dPt>
+          <dPt>
+            <idx val="9"/>
+            <spPr>
+              <a:solidFill>
+                <a:srgbClr val="3F51B5"/>
+              </a:solidFill>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </dPt>
           <cat>
             <numRef>
               <f>'Endpoint Breakdown'!$A$3:$A$12</f>
@@ -356,7 +500,7 @@
       <row>14</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="10080000" cy="5040000"/>
+    <ext cx="8640000" cy="5040000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="1" name="Chart 1"/>
@@ -660,17 +804,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="006C63FF"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E28"/>
+  <dimension ref="A1:G35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="5" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -679,133 +825,189 @@
           <t>AgriRent — K6 Baseline Load Test Report</t>
         </is>
       </c>
+      <c r="G1" s="2" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n"/>
+      <c r="B2" s="2" t="n"/>
+      <c r="C2" s="2" t="n"/>
+      <c r="D2" s="2" t="n"/>
+      <c r="E2" s="2" t="n"/>
+      <c r="F2" s="2" t="n"/>
+      <c r="G2" s="2" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>Report Generated</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>2026-06-18 13:14:28</t>
-        </is>
-      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-23 10:56:49</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="n"/>
+      <c r="D3" s="2" t="n"/>
+      <c r="E3" s="2" t="n"/>
+      <c r="F3" s="2" t="n"/>
+      <c r="G3" s="2" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Data Source</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>Simulated Baseline</t>
         </is>
       </c>
+      <c r="C4" s="2" t="n"/>
+      <c r="D4" s="2" t="n"/>
+      <c r="E4" s="2" t="n"/>
+      <c r="F4" s="2" t="n"/>
+      <c r="G4" s="2" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>Test Duration</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>1 minute (10s ramp-up / 40s hold / 10s ramp-down)</t>
         </is>
       </c>
+      <c r="C5" s="2" t="n"/>
+      <c r="D5" s="2" t="n"/>
+      <c r="E5" s="2" t="n"/>
+      <c r="F5" s="2" t="n"/>
+      <c r="G5" s="2" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="A6" s="3" t="inlineStr">
         <is>
           <t>Virtual Users (Peak)</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>100</t>
-        </is>
-      </c>
+      <c r="B6" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="C6" s="2" t="n"/>
+      <c r="D6" s="2" t="n"/>
+      <c r="E6" s="2" t="n"/>
+      <c r="F6" s="2" t="n"/>
+      <c r="G6" s="2" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>Target API</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>Supabase REST — atafeyidjdzedbktzivx.supabase.co</t>
         </is>
       </c>
+      <c r="C7" s="2" t="n"/>
+      <c r="D7" s="2" t="n"/>
+      <c r="E7" s="2" t="n"/>
+      <c r="F7" s="2" t="n"/>
+      <c r="G7" s="2" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n"/>
+      <c r="B8" s="2" t="n"/>
+      <c r="C8" s="2" t="n"/>
+      <c r="D8" s="2" t="n"/>
+      <c r="E8" s="2" t="n"/>
+      <c r="F8" s="2" t="n"/>
+      <c r="G8" s="2" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n"/>
+      <c r="B9" s="2" t="n"/>
+      <c r="C9" s="2" t="n"/>
+      <c r="D9" s="2" t="n"/>
+      <c r="E9" s="2" t="n"/>
+      <c r="F9" s="2" t="n"/>
+      <c r="G9" s="2" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="inlineStr">
+      <c r="A10" s="5" t="inlineStr">
         <is>
           <t>Key Performance Indicators</t>
         </is>
       </c>
+      <c r="G10" s="2" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="5" t="inlineStr">
+      <c r="A11" s="6" t="inlineStr">
         <is>
           <t>KPI</t>
         </is>
       </c>
-      <c r="B11" s="5" t="inlineStr">
+      <c r="B11" s="6" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
       </c>
-      <c r="C11" s="5" t="inlineStr">
+      <c r="C11" s="6" t="inlineStr">
         <is>
           <t>Unit</t>
         </is>
       </c>
-      <c r="D11" s="5" t="inlineStr">
+      <c r="D11" s="6" t="inlineStr">
         <is>
           <t>Threshold</t>
         </is>
       </c>
-      <c r="E11" s="5" t="inlineStr">
+      <c r="E11" s="6" t="inlineStr">
         <is>
           <t>Result</t>
         </is>
       </c>
+      <c r="F11" s="2" t="n"/>
+      <c r="G11" s="2" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="6" t="inlineStr">
+      <c r="A12" s="7" t="inlineStr">
         <is>
           <t>Total Requests</t>
         </is>
       </c>
-      <c r="B12" s="7" t="n">
+      <c r="B12" s="8" t="n">
         <v>7200</v>
       </c>
-      <c r="C12" s="7" t="inlineStr">
+      <c r="C12" s="9" t="inlineStr">
         <is>
           <t>count</t>
         </is>
       </c>
-      <c r="D12" s="7" t="inlineStr">
+      <c r="D12" s="9" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E12" s="7" t="inlineStr">
+      <c r="E12" s="10" t="inlineStr">
         <is>
           <t>INFO</t>
         </is>
       </c>
+      <c r="F12" s="2" t="n"/>
+      <c r="G12" s="2" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="8" t="inlineStr">
+      <c r="A13" s="7" t="inlineStr">
         <is>
           <t>Requests per Second</t>
         </is>
       </c>
-      <c r="B13" s="9" t="n">
+      <c r="B13" s="8" t="n">
         <v>120</v>
       </c>
       <c r="C13" s="9" t="inlineStr">
@@ -818,27 +1020,29 @@
           <t>&gt; 50</t>
         </is>
       </c>
-      <c r="E13" s="10" t="inlineStr">
+      <c r="E13" s="11" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
+      <c r="F13" s="2" t="n"/>
+      <c r="G13" s="2" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="6" t="inlineStr">
+      <c r="A14" s="7" t="inlineStr">
         <is>
           <t>Avg Response Time</t>
         </is>
       </c>
-      <c r="B14" s="7" t="n">
+      <c r="B14" s="8" t="n">
         <v>250</v>
       </c>
-      <c r="C14" s="7" t="inlineStr">
+      <c r="C14" s="9" t="inlineStr">
         <is>
           <t>ms</t>
         </is>
       </c>
-      <c r="D14" s="7" t="inlineStr">
+      <c r="D14" s="9" t="inlineStr">
         <is>
           <t>&lt; 500ms</t>
         </is>
@@ -848,14 +1052,16 @@
           <t>PASS</t>
         </is>
       </c>
+      <c r="F14" s="2" t="n"/>
+      <c r="G14" s="2" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="8" t="inlineStr">
+      <c r="A15" s="7" t="inlineStr">
         <is>
           <t>Min Response Time</t>
         </is>
       </c>
-      <c r="B15" s="9" t="n">
+      <c r="B15" s="8" t="n">
         <v>50</v>
       </c>
       <c r="C15" s="9" t="inlineStr">
@@ -868,27 +1074,29 @@
           <t>—</t>
         </is>
       </c>
-      <c r="E15" s="9" t="inlineStr">
+      <c r="E15" s="10" t="inlineStr">
         <is>
           <t>INFO</t>
         </is>
       </c>
+      <c r="F15" s="2" t="n"/>
+      <c r="G15" s="2" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="6" t="inlineStr">
+      <c r="A16" s="7" t="inlineStr">
         <is>
           <t>Max Response Time</t>
         </is>
       </c>
-      <c r="B16" s="7" t="n">
+      <c r="B16" s="8" t="n">
         <v>1500</v>
       </c>
-      <c r="C16" s="7" t="inlineStr">
+      <c r="C16" s="9" t="inlineStr">
         <is>
           <t>ms</t>
         </is>
       </c>
-      <c r="D16" s="7" t="inlineStr">
+      <c r="D16" s="9" t="inlineStr">
         <is>
           <t>&lt; 3000ms</t>
         </is>
@@ -898,14 +1106,16 @@
           <t>PASS</t>
         </is>
       </c>
+      <c r="F16" s="2" t="n"/>
+      <c r="G16" s="2" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="8" t="inlineStr">
+      <c r="A17" s="7" t="inlineStr">
         <is>
           <t>Median Response Time</t>
         </is>
       </c>
-      <c r="B17" s="9" t="n">
+      <c r="B17" s="8" t="n">
         <v>200</v>
       </c>
       <c r="C17" s="9" t="inlineStr">
@@ -918,27 +1128,29 @@
           <t>&lt; 400ms</t>
         </is>
       </c>
-      <c r="E17" s="10" t="inlineStr">
+      <c r="E17" s="11" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
+      <c r="F17" s="2" t="n"/>
+      <c r="G17" s="2" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="6" t="inlineStr">
+      <c r="A18" s="7" t="inlineStr">
         <is>
           <t>p(90) Response Time</t>
         </is>
       </c>
-      <c r="B18" s="7" t="n">
+      <c r="B18" s="8" t="n">
         <v>800</v>
       </c>
-      <c r="C18" s="7" t="inlineStr">
+      <c r="C18" s="9" t="inlineStr">
         <is>
           <t>ms</t>
         </is>
       </c>
-      <c r="D18" s="7" t="inlineStr">
+      <c r="D18" s="9" t="inlineStr">
         <is>
           <t>&lt; 1500ms</t>
         </is>
@@ -948,14 +1160,16 @@
           <t>PASS</t>
         </is>
       </c>
+      <c r="F18" s="2" t="n"/>
+      <c r="G18" s="2" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="8" t="inlineStr">
+      <c r="A19" s="7" t="inlineStr">
         <is>
           <t>p(95) Response Time</t>
         </is>
       </c>
-      <c r="B19" s="9" t="n">
+      <c r="B19" s="8" t="n">
         <v>1200</v>
       </c>
       <c r="C19" s="9" t="inlineStr">
@@ -968,27 +1182,29 @@
           <t>&lt; 2000ms</t>
         </is>
       </c>
-      <c r="E19" s="10" t="inlineStr">
+      <c r="E19" s="11" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
+      <c r="F19" s="2" t="n"/>
+      <c r="G19" s="2" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="6" t="inlineStr">
+      <c r="A20" s="7" t="inlineStr">
         <is>
           <t>Error Rate</t>
         </is>
       </c>
-      <c r="B20" s="7" t="n">
+      <c r="B20" s="8" t="n">
         <v>0.5</v>
       </c>
-      <c r="C20" s="7" t="inlineStr">
+      <c r="C20" s="9" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="D20" s="7" t="inlineStr">
+      <c r="D20" s="9" t="inlineStr">
         <is>
           <t>&lt; 10%</t>
         </is>
@@ -998,216 +1214,292 @@
           <t>PASS</t>
         </is>
       </c>
+      <c r="F20" s="2" t="n"/>
+      <c r="G20" s="2" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="8" t="inlineStr">
+      <c r="A21" s="2" t="n"/>
+      <c r="B21" s="2" t="n"/>
+      <c r="C21" s="2" t="n"/>
+      <c r="D21" s="2" t="n"/>
+      <c r="E21" s="2" t="n"/>
+      <c r="F21" s="2" t="n"/>
+      <c r="G21" s="2" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="7" t="inlineStr">
         <is>
           <t>Check Pass Rate</t>
         </is>
       </c>
-      <c r="B21" s="9" t="n">
+      <c r="B22" s="8" t="n">
         <v>99.5</v>
       </c>
-      <c r="C21" s="9" t="inlineStr">
+      <c r="C22" s="9" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="D21" s="9" t="inlineStr">
+      <c r="D22" s="9" t="inlineStr">
         <is>
           <t>&gt; 95%</t>
         </is>
       </c>
-      <c r="E21" s="10" t="inlineStr">
+      <c r="E22" s="11" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="6" t="inlineStr">
+      <c r="F22" s="2" t="n"/>
+      <c r="G22" s="2" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="7" t="inlineStr">
         <is>
           <t>Data Received</t>
         </is>
       </c>
-      <c r="B22" s="7" t="n">
-        <v>15</v>
-      </c>
-      <c r="C22" s="7" t="inlineStr">
+      <c r="B23" s="8" t="n">
+        <v>12</v>
+      </c>
+      <c r="C23" s="9" t="inlineStr">
         <is>
           <t>MB</t>
         </is>
       </c>
-      <c r="D22" s="7" t="inlineStr">
+      <c r="D23" s="9" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E22" s="7" t="inlineStr">
+      <c r="E23" s="10" t="inlineStr">
         <is>
           <t>INFO</t>
         </is>
       </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="8" t="inlineStr">
+      <c r="F23" s="2" t="n"/>
+      <c r="G23" s="2" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="7" t="inlineStr">
         <is>
           <t>Data Sent</t>
         </is>
       </c>
-      <c r="B23" s="9" t="n">
+      <c r="B24" s="8" t="n">
         <v>3.2</v>
       </c>
-      <c r="C23" s="9" t="inlineStr">
+      <c r="C24" s="9" t="inlineStr">
         <is>
           <t>MB</t>
         </is>
       </c>
-      <c r="D23" s="9" t="inlineStr">
+      <c r="D24" s="9" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E23" s="9" t="inlineStr">
+      <c r="E24" s="10" t="inlineStr">
         <is>
           <t>INFO</t>
         </is>
       </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="6" t="inlineStr">
+      <c r="F24" s="2" t="n"/>
+      <c r="G24" s="2" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="7" t="inlineStr">
         <is>
           <t>Avg Connection Time</t>
         </is>
       </c>
-      <c r="B24" s="7" t="n">
+      <c r="B25" s="8" t="n">
         <v>12.5</v>
       </c>
-      <c r="C24" s="7" t="inlineStr">
+      <c r="C25" s="9" t="inlineStr">
         <is>
           <t>ms</t>
         </is>
       </c>
-      <c r="D24" s="7" t="inlineStr">
+      <c r="D25" s="9" t="inlineStr">
         <is>
           <t>&lt; 100ms</t>
         </is>
       </c>
-      <c r="E24" s="11" t="inlineStr">
+      <c r="E25" s="11" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="8" t="inlineStr">
+      <c r="F25" s="2" t="n"/>
+      <c r="G25" s="2" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="7" t="inlineStr">
         <is>
           <t>Avg TLS Handshake</t>
         </is>
       </c>
-      <c r="B25" s="9" t="n">
+      <c r="B26" s="8" t="n">
         <v>45</v>
       </c>
-      <c r="C25" s="9" t="inlineStr">
+      <c r="C26" s="9" t="inlineStr">
         <is>
           <t>ms</t>
         </is>
       </c>
-      <c r="D25" s="9" t="inlineStr">
+      <c r="D26" s="9" t="inlineStr">
         <is>
           <t>&lt; 200ms</t>
         </is>
       </c>
-      <c r="E25" s="10" t="inlineStr">
+      <c r="E26" s="11" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="6" t="inlineStr">
+      <c r="F26" s="2" t="n"/>
+      <c r="G26" s="2" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="7" t="inlineStr">
         <is>
           <t>Avg Waiting (TTFB)</t>
         </is>
       </c>
-      <c r="B26" s="7" t="n">
+      <c r="B27" s="8" t="n">
         <v>180</v>
       </c>
-      <c r="C26" s="7" t="inlineStr">
+      <c r="C27" s="9" t="inlineStr">
         <is>
           <t>ms</t>
         </is>
       </c>
-      <c r="D26" s="7" t="inlineStr">
+      <c r="D27" s="9" t="inlineStr">
         <is>
           <t>&lt; 400ms</t>
         </is>
       </c>
-      <c r="E26" s="11" t="inlineStr">
+      <c r="E27" s="11" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="8" t="inlineStr">
+      <c r="F27" s="2" t="n"/>
+      <c r="G27" s="2" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="7" t="inlineStr">
         <is>
           <t>Total Iterations</t>
         </is>
       </c>
-      <c r="B27" s="9" t="n">
+      <c r="B28" s="8" t="n">
         <v>720</v>
       </c>
-      <c r="C27" s="9" t="inlineStr">
+      <c r="C28" s="9" t="inlineStr">
         <is>
           <t>count</t>
         </is>
       </c>
-      <c r="D27" s="9" t="inlineStr">
+      <c r="D28" s="9" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E27" s="9" t="inlineStr">
+      <c r="E28" s="10" t="inlineStr">
         <is>
           <t>INFO</t>
         </is>
       </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="6" t="inlineStr">
+      <c r="F28" s="2" t="n"/>
+      <c r="G28" s="2" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="7" t="inlineStr">
         <is>
           <t>Iterations per Second</t>
         </is>
       </c>
-      <c r="B28" s="7" t="n">
+      <c r="B29" s="8" t="n">
         <v>12</v>
       </c>
-      <c r="C28" s="7" t="inlineStr">
+      <c r="C29" s="9" t="inlineStr">
         <is>
           <t>iter/s</t>
         </is>
       </c>
-      <c r="D28" s="7" t="inlineStr">
+      <c r="D29" s="9" t="inlineStr">
         <is>
           <t>&gt; 5</t>
         </is>
       </c>
-      <c r="E28" s="11" t="inlineStr">
+      <c r="E29" s="11" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
+      <c r="F29" s="2" t="n"/>
+      <c r="G29" s="2" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="n"/>
+      <c r="B30" s="2" t="n"/>
+      <c r="C30" s="2" t="n"/>
+      <c r="D30" s="2" t="n"/>
+      <c r="E30" s="2" t="n"/>
+      <c r="F30" s="2" t="n"/>
+      <c r="G30" s="2" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="n"/>
+      <c r="B31" s="2" t="n"/>
+      <c r="C31" s="2" t="n"/>
+      <c r="D31" s="2" t="n"/>
+      <c r="E31" s="2" t="n"/>
+      <c r="F31" s="2" t="n"/>
+      <c r="G31" s="2" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="n"/>
+      <c r="B32" s="2" t="n"/>
+      <c r="C32" s="2" t="n"/>
+      <c r="D32" s="2" t="n"/>
+      <c r="E32" s="2" t="n"/>
+      <c r="F32" s="2" t="n"/>
+      <c r="G32" s="2" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="n"/>
+      <c r="B33" s="2" t="n"/>
+      <c r="C33" s="2" t="n"/>
+      <c r="D33" s="2" t="n"/>
+      <c r="E33" s="2" t="n"/>
+      <c r="F33" s="2" t="n"/>
+      <c r="G33" s="2" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="n"/>
+      <c r="B34" s="2" t="n"/>
+      <c r="C34" s="2" t="n"/>
+      <c r="D34" s="2" t="n"/>
+      <c r="E34" s="2" t="n"/>
+      <c r="F34" s="2" t="n"/>
+      <c r="G34" s="2" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="n"/>
+      <c r="B35" s="2" t="n"/>
+      <c r="C35" s="2" t="n"/>
+      <c r="D35" s="2" t="n"/>
+      <c r="E35" s="2" t="n"/>
+      <c r="F35" s="2" t="n"/>
+      <c r="G35" s="2" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="7">
-    <mergeCell ref="B4:E4"/>
-    <mergeCell ref="A10:E10"/>
-    <mergeCell ref="B6:E6"/>
-    <mergeCell ref="B7:E7"/>
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="B3:E3"/>
-    <mergeCell ref="B5:E5"/>
+  <mergeCells count="2">
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A10:F10"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1216,19 +1508,20 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="0000BCD4"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:H65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1237,46 +1530,48 @@
           <t>Per-Endpoint Load Test Results</t>
         </is>
       </c>
+      <c r="H1" s="2" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" s="13" t="inlineStr">
+      <c r="A2" s="6" t="inlineStr">
         <is>
           <t>Endpoint</t>
         </is>
       </c>
-      <c r="B2" s="13" t="inlineStr">
+      <c r="B2" s="6" t="inlineStr">
         <is>
           <t>Method</t>
         </is>
       </c>
-      <c r="C2" s="13" t="inlineStr">
+      <c r="C2" s="6" t="inlineStr">
         <is>
           <t>Requests</t>
         </is>
       </c>
-      <c r="D2" s="13" t="inlineStr">
-        <is>
-          <t>Avg (ms)</t>
-        </is>
-      </c>
-      <c r="E2" s="13" t="inlineStr">
-        <is>
-          <t>Min (ms)</t>
-        </is>
-      </c>
-      <c r="F2" s="13" t="inlineStr">
-        <is>
-          <t>Max (ms)</t>
-        </is>
-      </c>
-      <c r="G2" s="13" t="inlineStr">
+      <c r="D2" s="6" t="inlineStr">
+        <is>
+          <t>Avg(ms)</t>
+        </is>
+      </c>
+      <c r="E2" s="6" t="inlineStr">
+        <is>
+          <t>Min(ms)</t>
+        </is>
+      </c>
+      <c r="F2" s="6" t="inlineStr">
+        <is>
+          <t>Max(ms)</t>
+        </is>
+      </c>
+      <c r="G2" s="6" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
+      <c r="H2" s="2" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="9" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>GET /vehicles</t>
         </is>
@@ -1287,56 +1582,58 @@
         </is>
       </c>
       <c r="C3" s="9" t="n">
-        <v>1080</v>
-      </c>
-      <c r="D3" s="9" t="n">
+        <v>720</v>
+      </c>
+      <c r="D3" s="8" t="n">
         <v>225</v>
       </c>
       <c r="E3" s="9" t="n">
-        <v>50</v>
+        <v>5</v>
       </c>
       <c r="F3" s="9" t="n">
-        <v>1200</v>
-      </c>
-      <c r="G3" s="10" t="inlineStr">
+        <v>1500</v>
+      </c>
+      <c r="G3" s="13" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
+      <c r="H3" s="2" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="7" t="inlineStr">
-        <is>
-          <t>GET /vehicles?filter</t>
-        </is>
-      </c>
-      <c r="B4" s="7" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>GET /vehiclesFilter</t>
+        </is>
+      </c>
+      <c r="B4" s="9" t="inlineStr">
         <is>
           <t>GET</t>
         </is>
       </c>
-      <c r="C4" s="7" t="n">
-        <v>864</v>
-      </c>
-      <c r="D4" s="7" t="n">
-        <v>275</v>
-      </c>
-      <c r="E4" s="7" t="n">
-        <v>60</v>
-      </c>
-      <c r="F4" s="7" t="n">
-        <v>1350</v>
-      </c>
-      <c r="G4" s="11" t="inlineStr">
+      <c r="C4" s="9" t="n">
+        <v>720</v>
+      </c>
+      <c r="D4" s="8" t="n">
+        <v>98.40000000000001</v>
+      </c>
+      <c r="E4" s="9" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="F4" s="9" t="n">
+        <v>1500</v>
+      </c>
+      <c r="G4" s="13" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
+      <c r="H4" s="2" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="9" t="inlineStr">
-        <is>
-          <t>GET /vehicles/:id</t>
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>GET /vehicleSorted</t>
         </is>
       </c>
       <c r="B5" s="9" t="inlineStr">
@@ -1347,52 +1644,54 @@
       <c r="C5" s="9" t="n">
         <v>720</v>
       </c>
-      <c r="D5" s="9" t="n">
-        <v>175</v>
+      <c r="D5" s="8" t="n">
+        <v>74</v>
       </c>
       <c r="E5" s="9" t="n">
-        <v>40</v>
+        <v>4</v>
       </c>
       <c r="F5" s="9" t="n">
-        <v>900</v>
-      </c>
-      <c r="G5" s="10" t="inlineStr">
+        <v>520</v>
+      </c>
+      <c r="G5" s="13" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
+      <c r="H5" s="2" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="inlineStr">
+      <c r="A6" s="3" t="inlineStr">
         <is>
           <t>GET /bookings</t>
         </is>
       </c>
-      <c r="B6" s="7" t="inlineStr">
+      <c r="B6" s="9" t="inlineStr">
         <is>
           <t>GET</t>
         </is>
       </c>
-      <c r="C6" s="7" t="n">
+      <c r="C6" s="9" t="n">
         <v>720</v>
       </c>
-      <c r="D6" s="7" t="n">
-        <v>250</v>
-      </c>
-      <c r="E6" s="7" t="n">
-        <v>50</v>
-      </c>
-      <c r="F6" s="7" t="n">
+      <c r="D6" s="8" t="n">
+        <v>200</v>
+      </c>
+      <c r="E6" s="9" t="n">
+        <v>10</v>
+      </c>
+      <c r="F6" s="9" t="n">
         <v>1275</v>
       </c>
-      <c r="G6" s="11" t="inlineStr">
+      <c r="G6" s="13" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
+      <c r="H6" s="2" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="9" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>GET /users</t>
         </is>
@@ -1405,52 +1704,54 @@
       <c r="C7" s="9" t="n">
         <v>720</v>
       </c>
-      <c r="D7" s="9" t="n">
+      <c r="D7" s="8" t="n">
         <v>237.5</v>
       </c>
       <c r="E7" s="9" t="n">
-        <v>55</v>
+        <v>5</v>
       </c>
       <c r="F7" s="9" t="n">
-        <v>1050</v>
-      </c>
-      <c r="G7" s="10" t="inlineStr">
+        <v>670</v>
+      </c>
+      <c r="G7" s="13" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
+      <c r="H7" s="2" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="inlineStr">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>GET /reviews</t>
         </is>
       </c>
-      <c r="B8" s="7" t="inlineStr">
+      <c r="B8" s="9" t="inlineStr">
         <is>
           <t>GET</t>
         </is>
       </c>
-      <c r="C8" s="7" t="n">
-        <v>576</v>
-      </c>
-      <c r="D8" s="7" t="n">
-        <v>212.5</v>
-      </c>
-      <c r="E8" s="7" t="n">
+      <c r="C8" s="9" t="n">
+        <v>575</v>
+      </c>
+      <c r="D8" s="8" t="n">
+        <v>131.5</v>
+      </c>
+      <c r="E8" s="9" t="n">
         <v>45</v>
       </c>
-      <c r="F8" s="7" t="n">
+      <c r="F8" s="9" t="n">
         <v>975</v>
       </c>
-      <c r="G8" s="11" t="inlineStr">
+      <c r="G8" s="13" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
+      <c r="H8" s="2" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="9" t="inlineStr">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t>GET /payments</t>
         </is>
@@ -1461,56 +1762,58 @@
         </is>
       </c>
       <c r="C9" s="9" t="n">
-        <v>576</v>
-      </c>
-      <c r="D9" s="9" t="n">
+        <v>575</v>
+      </c>
+      <c r="D9" s="8" t="n">
         <v>262.5</v>
       </c>
       <c r="E9" s="9" t="n">
-        <v>65</v>
+        <v>40</v>
       </c>
       <c r="F9" s="9" t="n">
-        <v>1350</v>
-      </c>
-      <c r="G9" s="10" t="inlineStr">
+        <v>1170</v>
+      </c>
+      <c r="G9" s="13" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
+      <c r="H9" s="2" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="7" t="inlineStr">
+      <c r="A10" s="3" t="inlineStr">
         <is>
           <t>GET /notifications</t>
         </is>
       </c>
-      <c r="B10" s="7" t="inlineStr">
+      <c r="B10" s="9" t="inlineStr">
         <is>
           <t>GET</t>
         </is>
       </c>
-      <c r="C10" s="7" t="n">
-        <v>576</v>
-      </c>
-      <c r="D10" s="7" t="n">
-        <v>200</v>
-      </c>
-      <c r="E10" s="7" t="n">
+      <c r="C10" s="9" t="n">
+        <v>575</v>
+      </c>
+      <c r="D10" s="8" t="n">
+        <v>300</v>
+      </c>
+      <c r="E10" s="9" t="n">
         <v>50</v>
       </c>
-      <c r="F10" s="7" t="n">
-        <v>750</v>
-      </c>
-      <c r="G10" s="11" t="inlineStr">
+      <c r="F10" s="9" t="n">
+        <v>770</v>
+      </c>
+      <c r="G10" s="13" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
+      <c r="H10" s="2" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="9" t="inlineStr">
-        <is>
-          <t>GET /vehicles?sorted</t>
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>GET /vehiclesSorted</t>
         </is>
       </c>
       <c r="B11" s="9" t="inlineStr">
@@ -1521,49 +1824,581 @@
       <c r="C11" s="9" t="n">
         <v>720</v>
       </c>
-      <c r="D11" s="9" t="n">
+      <c r="D11" s="8" t="n">
         <v>300</v>
       </c>
       <c r="E11" s="9" t="n">
         <v>75</v>
       </c>
       <c r="F11" s="9" t="n">
-        <v>1650</v>
-      </c>
-      <c r="G11" s="10" t="inlineStr">
+        <v>850</v>
+      </c>
+      <c r="G11" s="13" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
+      <c r="H11" s="2" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="7" t="inlineStr">
-        <is>
-          <t>GET /bookings?status</t>
-        </is>
-      </c>
-      <c r="B12" s="7" t="inlineStr">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>GET /bookingsPending</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="inlineStr">
         <is>
           <t>GET</t>
         </is>
       </c>
-      <c r="C12" s="7" t="n">
-        <v>648</v>
-      </c>
-      <c r="D12" s="7" t="n">
+      <c r="C12" s="9" t="n">
+        <v>645</v>
+      </c>
+      <c r="D12" s="8" t="n">
         <v>287.5</v>
       </c>
-      <c r="E12" s="7" t="n">
+      <c r="E12" s="9" t="n">
         <v>60</v>
       </c>
-      <c r="F12" s="7" t="n">
-        <v>1425</v>
-      </c>
-      <c r="G12" s="11" t="inlineStr">
+      <c r="F12" s="9" t="n">
+        <v>1455</v>
+      </c>
+      <c r="G12" s="13" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
+      <c r="H12" s="2" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n"/>
+      <c r="B13" s="2" t="n"/>
+      <c r="C13" s="2" t="n"/>
+      <c r="D13" s="2" t="n"/>
+      <c r="E13" s="2" t="n"/>
+      <c r="F13" s="2" t="n"/>
+      <c r="G13" s="2" t="n"/>
+      <c r="H13" s="2" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n"/>
+      <c r="B14" s="2" t="n"/>
+      <c r="C14" s="2" t="n"/>
+      <c r="D14" s="2" t="n"/>
+      <c r="E14" s="2" t="n"/>
+      <c r="F14" s="2" t="n"/>
+      <c r="G14" s="2" t="n"/>
+      <c r="H14" s="2" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n"/>
+      <c r="B15" s="2" t="n"/>
+      <c r="C15" s="2" t="n"/>
+      <c r="D15" s="2" t="n"/>
+      <c r="E15" s="2" t="n"/>
+      <c r="F15" s="2" t="n"/>
+      <c r="G15" s="2" t="n"/>
+      <c r="H15" s="2" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n"/>
+      <c r="B16" s="2" t="n"/>
+      <c r="C16" s="2" t="n"/>
+      <c r="D16" s="2" t="n"/>
+      <c r="E16" s="2" t="n"/>
+      <c r="F16" s="2" t="n"/>
+      <c r="G16" s="2" t="n"/>
+      <c r="H16" s="2" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n"/>
+      <c r="B17" s="2" t="n"/>
+      <c r="C17" s="2" t="n"/>
+      <c r="D17" s="2" t="n"/>
+      <c r="E17" s="2" t="n"/>
+      <c r="F17" s="2" t="n"/>
+      <c r="G17" s="2" t="n"/>
+      <c r="H17" s="2" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n"/>
+      <c r="B18" s="2" t="n"/>
+      <c r="C18" s="2" t="n"/>
+      <c r="D18" s="2" t="n"/>
+      <c r="E18" s="2" t="n"/>
+      <c r="F18" s="2" t="n"/>
+      <c r="G18" s="2" t="n"/>
+      <c r="H18" s="2" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="n"/>
+      <c r="B19" s="2" t="n"/>
+      <c r="C19" s="2" t="n"/>
+      <c r="D19" s="2" t="n"/>
+      <c r="E19" s="2" t="n"/>
+      <c r="F19" s="2" t="n"/>
+      <c r="G19" s="2" t="n"/>
+      <c r="H19" s="2" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="n"/>
+      <c r="B20" s="2" t="n"/>
+      <c r="C20" s="2" t="n"/>
+      <c r="D20" s="2" t="n"/>
+      <c r="E20" s="2" t="n"/>
+      <c r="F20" s="2" t="n"/>
+      <c r="G20" s="2" t="n"/>
+      <c r="H20" s="2" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="n"/>
+      <c r="B21" s="2" t="n"/>
+      <c r="C21" s="2" t="n"/>
+      <c r="D21" s="2" t="n"/>
+      <c r="E21" s="2" t="n"/>
+      <c r="F21" s="2" t="n"/>
+      <c r="G21" s="2" t="n"/>
+      <c r="H21" s="2" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="n"/>
+      <c r="B22" s="2" t="n"/>
+      <c r="C22" s="2" t="n"/>
+      <c r="D22" s="2" t="n"/>
+      <c r="E22" s="2" t="n"/>
+      <c r="F22" s="2" t="n"/>
+      <c r="G22" s="2" t="n"/>
+      <c r="H22" s="2" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="n"/>
+      <c r="B23" s="2" t="n"/>
+      <c r="C23" s="2" t="n"/>
+      <c r="D23" s="2" t="n"/>
+      <c r="E23" s="2" t="n"/>
+      <c r="F23" s="2" t="n"/>
+      <c r="G23" s="2" t="n"/>
+      <c r="H23" s="2" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="n"/>
+      <c r="B24" s="2" t="n"/>
+      <c r="C24" s="2" t="n"/>
+      <c r="D24" s="2" t="n"/>
+      <c r="E24" s="2" t="n"/>
+      <c r="F24" s="2" t="n"/>
+      <c r="G24" s="2" t="n"/>
+      <c r="H24" s="2" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="n"/>
+      <c r="B25" s="2" t="n"/>
+      <c r="C25" s="2" t="n"/>
+      <c r="D25" s="2" t="n"/>
+      <c r="E25" s="2" t="n"/>
+      <c r="F25" s="2" t="n"/>
+      <c r="G25" s="2" t="n"/>
+      <c r="H25" s="2" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="n"/>
+      <c r="B26" s="2" t="n"/>
+      <c r="C26" s="2" t="n"/>
+      <c r="D26" s="2" t="n"/>
+      <c r="E26" s="2" t="n"/>
+      <c r="F26" s="2" t="n"/>
+      <c r="G26" s="2" t="n"/>
+      <c r="H26" s="2" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="n"/>
+      <c r="B27" s="2" t="n"/>
+      <c r="C27" s="2" t="n"/>
+      <c r="D27" s="2" t="n"/>
+      <c r="E27" s="2" t="n"/>
+      <c r="F27" s="2" t="n"/>
+      <c r="G27" s="2" t="n"/>
+      <c r="H27" s="2" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="n"/>
+      <c r="B28" s="2" t="n"/>
+      <c r="C28" s="2" t="n"/>
+      <c r="D28" s="2" t="n"/>
+      <c r="E28" s="2" t="n"/>
+      <c r="F28" s="2" t="n"/>
+      <c r="G28" s="2" t="n"/>
+      <c r="H28" s="2" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="n"/>
+      <c r="B29" s="2" t="n"/>
+      <c r="C29" s="2" t="n"/>
+      <c r="D29" s="2" t="n"/>
+      <c r="E29" s="2" t="n"/>
+      <c r="F29" s="2" t="n"/>
+      <c r="G29" s="2" t="n"/>
+      <c r="H29" s="2" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="n"/>
+      <c r="B30" s="2" t="n"/>
+      <c r="C30" s="2" t="n"/>
+      <c r="D30" s="2" t="n"/>
+      <c r="E30" s="2" t="n"/>
+      <c r="F30" s="2" t="n"/>
+      <c r="G30" s="2" t="n"/>
+      <c r="H30" s="2" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="n"/>
+      <c r="B31" s="2" t="n"/>
+      <c r="C31" s="2" t="n"/>
+      <c r="D31" s="2" t="n"/>
+      <c r="E31" s="2" t="n"/>
+      <c r="F31" s="2" t="n"/>
+      <c r="G31" s="2" t="n"/>
+      <c r="H31" s="2" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="n"/>
+      <c r="B32" s="2" t="n"/>
+      <c r="C32" s="2" t="n"/>
+      <c r="D32" s="2" t="n"/>
+      <c r="E32" s="2" t="n"/>
+      <c r="F32" s="2" t="n"/>
+      <c r="G32" s="2" t="n"/>
+      <c r="H32" s="2" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="n"/>
+      <c r="B33" s="2" t="n"/>
+      <c r="C33" s="2" t="n"/>
+      <c r="D33" s="2" t="n"/>
+      <c r="E33" s="2" t="n"/>
+      <c r="F33" s="2" t="n"/>
+      <c r="G33" s="2" t="n"/>
+      <c r="H33" s="2" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="n"/>
+      <c r="B34" s="2" t="n"/>
+      <c r="C34" s="2" t="n"/>
+      <c r="D34" s="2" t="n"/>
+      <c r="E34" s="2" t="n"/>
+      <c r="F34" s="2" t="n"/>
+      <c r="G34" s="2" t="n"/>
+      <c r="H34" s="2" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="n"/>
+      <c r="B35" s="2" t="n"/>
+      <c r="C35" s="2" t="n"/>
+      <c r="D35" s="2" t="n"/>
+      <c r="E35" s="2" t="n"/>
+      <c r="F35" s="2" t="n"/>
+      <c r="G35" s="2" t="n"/>
+      <c r="H35" s="2" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="n"/>
+      <c r="B36" s="2" t="n"/>
+      <c r="C36" s="2" t="n"/>
+      <c r="D36" s="2" t="n"/>
+      <c r="E36" s="2" t="n"/>
+      <c r="F36" s="2" t="n"/>
+      <c r="G36" s="2" t="n"/>
+      <c r="H36" s="2" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="n"/>
+      <c r="B37" s="2" t="n"/>
+      <c r="C37" s="2" t="n"/>
+      <c r="D37" s="2" t="n"/>
+      <c r="E37" s="2" t="n"/>
+      <c r="F37" s="2" t="n"/>
+      <c r="G37" s="2" t="n"/>
+      <c r="H37" s="2" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="n"/>
+      <c r="B38" s="2" t="n"/>
+      <c r="C38" s="2" t="n"/>
+      <c r="D38" s="2" t="n"/>
+      <c r="E38" s="2" t="n"/>
+      <c r="F38" s="2" t="n"/>
+      <c r="G38" s="2" t="n"/>
+      <c r="H38" s="2" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="n"/>
+      <c r="B39" s="2" t="n"/>
+      <c r="C39" s="2" t="n"/>
+      <c r="D39" s="2" t="n"/>
+      <c r="E39" s="2" t="n"/>
+      <c r="F39" s="2" t="n"/>
+      <c r="G39" s="2" t="n"/>
+      <c r="H39" s="2" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="n"/>
+      <c r="B40" s="2" t="n"/>
+      <c r="C40" s="2" t="n"/>
+      <c r="D40" s="2" t="n"/>
+      <c r="E40" s="2" t="n"/>
+      <c r="F40" s="2" t="n"/>
+      <c r="G40" s="2" t="n"/>
+      <c r="H40" s="2" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="n"/>
+      <c r="B41" s="2" t="n"/>
+      <c r="C41" s="2" t="n"/>
+      <c r="D41" s="2" t="n"/>
+      <c r="E41" s="2" t="n"/>
+      <c r="F41" s="2" t="n"/>
+      <c r="G41" s="2" t="n"/>
+      <c r="H41" s="2" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="n"/>
+      <c r="B42" s="2" t="n"/>
+      <c r="C42" s="2" t="n"/>
+      <c r="D42" s="2" t="n"/>
+      <c r="E42" s="2" t="n"/>
+      <c r="F42" s="2" t="n"/>
+      <c r="G42" s="2" t="n"/>
+      <c r="H42" s="2" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="n"/>
+      <c r="B43" s="2" t="n"/>
+      <c r="C43" s="2" t="n"/>
+      <c r="D43" s="2" t="n"/>
+      <c r="E43" s="2" t="n"/>
+      <c r="F43" s="2" t="n"/>
+      <c r="G43" s="2" t="n"/>
+      <c r="H43" s="2" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="n"/>
+      <c r="B44" s="2" t="n"/>
+      <c r="C44" s="2" t="n"/>
+      <c r="D44" s="2" t="n"/>
+      <c r="E44" s="2" t="n"/>
+      <c r="F44" s="2" t="n"/>
+      <c r="G44" s="2" t="n"/>
+      <c r="H44" s="2" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="n"/>
+      <c r="B45" s="2" t="n"/>
+      <c r="C45" s="2" t="n"/>
+      <c r="D45" s="2" t="n"/>
+      <c r="E45" s="2" t="n"/>
+      <c r="F45" s="2" t="n"/>
+      <c r="G45" s="2" t="n"/>
+      <c r="H45" s="2" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="n"/>
+      <c r="B46" s="2" t="n"/>
+      <c r="C46" s="2" t="n"/>
+      <c r="D46" s="2" t="n"/>
+      <c r="E46" s="2" t="n"/>
+      <c r="F46" s="2" t="n"/>
+      <c r="G46" s="2" t="n"/>
+      <c r="H46" s="2" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="n"/>
+      <c r="B47" s="2" t="n"/>
+      <c r="C47" s="2" t="n"/>
+      <c r="D47" s="2" t="n"/>
+      <c r="E47" s="2" t="n"/>
+      <c r="F47" s="2" t="n"/>
+      <c r="G47" s="2" t="n"/>
+      <c r="H47" s="2" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="n"/>
+      <c r="B48" s="2" t="n"/>
+      <c r="C48" s="2" t="n"/>
+      <c r="D48" s="2" t="n"/>
+      <c r="E48" s="2" t="n"/>
+      <c r="F48" s="2" t="n"/>
+      <c r="G48" s="2" t="n"/>
+      <c r="H48" s="2" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="n"/>
+      <c r="B49" s="2" t="n"/>
+      <c r="C49" s="2" t="n"/>
+      <c r="D49" s="2" t="n"/>
+      <c r="E49" s="2" t="n"/>
+      <c r="F49" s="2" t="n"/>
+      <c r="G49" s="2" t="n"/>
+      <c r="H49" s="2" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="n"/>
+      <c r="B50" s="2" t="n"/>
+      <c r="C50" s="2" t="n"/>
+      <c r="D50" s="2" t="n"/>
+      <c r="E50" s="2" t="n"/>
+      <c r="F50" s="2" t="n"/>
+      <c r="G50" s="2" t="n"/>
+      <c r="H50" s="2" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="n"/>
+      <c r="B51" s="2" t="n"/>
+      <c r="C51" s="2" t="n"/>
+      <c r="D51" s="2" t="n"/>
+      <c r="E51" s="2" t="n"/>
+      <c r="F51" s="2" t="n"/>
+      <c r="G51" s="2" t="n"/>
+      <c r="H51" s="2" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="n"/>
+      <c r="B52" s="2" t="n"/>
+      <c r="C52" s="2" t="n"/>
+      <c r="D52" s="2" t="n"/>
+      <c r="E52" s="2" t="n"/>
+      <c r="F52" s="2" t="n"/>
+      <c r="G52" s="2" t="n"/>
+      <c r="H52" s="2" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="n"/>
+      <c r="B53" s="2" t="n"/>
+      <c r="C53" s="2" t="n"/>
+      <c r="D53" s="2" t="n"/>
+      <c r="E53" s="2" t="n"/>
+      <c r="F53" s="2" t="n"/>
+      <c r="G53" s="2" t="n"/>
+      <c r="H53" s="2" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="n"/>
+      <c r="B54" s="2" t="n"/>
+      <c r="C54" s="2" t="n"/>
+      <c r="D54" s="2" t="n"/>
+      <c r="E54" s="2" t="n"/>
+      <c r="F54" s="2" t="n"/>
+      <c r="G54" s="2" t="n"/>
+      <c r="H54" s="2" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="n"/>
+      <c r="B55" s="2" t="n"/>
+      <c r="C55" s="2" t="n"/>
+      <c r="D55" s="2" t="n"/>
+      <c r="E55" s="2" t="n"/>
+      <c r="F55" s="2" t="n"/>
+      <c r="G55" s="2" t="n"/>
+      <c r="H55" s="2" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="n"/>
+      <c r="B56" s="2" t="n"/>
+      <c r="C56" s="2" t="n"/>
+      <c r="D56" s="2" t="n"/>
+      <c r="E56" s="2" t="n"/>
+      <c r="F56" s="2" t="n"/>
+      <c r="G56" s="2" t="n"/>
+      <c r="H56" s="2" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="n"/>
+      <c r="B57" s="2" t="n"/>
+      <c r="C57" s="2" t="n"/>
+      <c r="D57" s="2" t="n"/>
+      <c r="E57" s="2" t="n"/>
+      <c r="F57" s="2" t="n"/>
+      <c r="G57" s="2" t="n"/>
+      <c r="H57" s="2" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="n"/>
+      <c r="B58" s="2" t="n"/>
+      <c r="C58" s="2" t="n"/>
+      <c r="D58" s="2" t="n"/>
+      <c r="E58" s="2" t="n"/>
+      <c r="F58" s="2" t="n"/>
+      <c r="G58" s="2" t="n"/>
+      <c r="H58" s="2" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="n"/>
+      <c r="B59" s="2" t="n"/>
+      <c r="C59" s="2" t="n"/>
+      <c r="D59" s="2" t="n"/>
+      <c r="E59" s="2" t="n"/>
+      <c r="F59" s="2" t="n"/>
+      <c r="G59" s="2" t="n"/>
+      <c r="H59" s="2" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="n"/>
+      <c r="B60" s="2" t="n"/>
+      <c r="C60" s="2" t="n"/>
+      <c r="D60" s="2" t="n"/>
+      <c r="E60" s="2" t="n"/>
+      <c r="F60" s="2" t="n"/>
+      <c r="G60" s="2" t="n"/>
+      <c r="H60" s="2" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="n"/>
+      <c r="B61" s="2" t="n"/>
+      <c r="C61" s="2" t="n"/>
+      <c r="D61" s="2" t="n"/>
+      <c r="E61" s="2" t="n"/>
+      <c r="F61" s="2" t="n"/>
+      <c r="G61" s="2" t="n"/>
+      <c r="H61" s="2" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="n"/>
+      <c r="B62" s="2" t="n"/>
+      <c r="C62" s="2" t="n"/>
+      <c r="D62" s="2" t="n"/>
+      <c r="E62" s="2" t="n"/>
+      <c r="F62" s="2" t="n"/>
+      <c r="G62" s="2" t="n"/>
+      <c r="H62" s="2" t="n"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="n"/>
+      <c r="B63" s="2" t="n"/>
+      <c r="C63" s="2" t="n"/>
+      <c r="D63" s="2" t="n"/>
+      <c r="E63" s="2" t="n"/>
+      <c r="F63" s="2" t="n"/>
+      <c r="G63" s="2" t="n"/>
+      <c r="H63" s="2" t="n"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="n"/>
+      <c r="B64" s="2" t="n"/>
+      <c r="C64" s="2" t="n"/>
+      <c r="D64" s="2" t="n"/>
+      <c r="E64" s="2" t="n"/>
+      <c r="F64" s="2" t="n"/>
+      <c r="G64" s="2" t="n"/>
+      <c r="H64" s="2" t="n"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="n"/>
+      <c r="B65" s="2" t="n"/>
+      <c r="C65" s="2" t="n"/>
+      <c r="D65" s="2" t="n"/>
+      <c r="E65" s="2" t="n"/>
+      <c r="F65" s="2" t="n"/>
+      <c r="G65" s="2" t="n"/>
+      <c r="H65" s="2" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1577,10 +2412,11 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="00FF9800"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B18"/>
+  <dimension ref="A1:D25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1593,198 +2429,280 @@
           <t>Load Test Configuration</t>
         </is>
       </c>
+      <c r="C1" s="2" t="n"/>
+      <c r="D1" s="2" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n"/>
+      <c r="B2" s="2" t="n"/>
+      <c r="C2" s="2" t="n"/>
+      <c r="D2" s="2" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="15" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>Tool</t>
         </is>
       </c>
-      <c r="B3" s="16" t="inlineStr">
+      <c r="B3" s="4" t="inlineStr">
         <is>
           <t>Grafana k6 (v0.50+)</t>
         </is>
       </c>
+      <c r="C3" s="2" t="n"/>
+      <c r="D3" s="2" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="17" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Test Type</t>
         </is>
       </c>
-      <c r="B4" s="18" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>Baseline / Load Test</t>
         </is>
       </c>
+      <c r="C4" s="2" t="n"/>
+      <c r="D4" s="2" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="15" t="inlineStr">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>Protocol</t>
         </is>
       </c>
-      <c r="B5" s="16" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>HTTPS (REST API)</t>
         </is>
       </c>
+      <c r="C5" s="2" t="n"/>
+      <c r="D5" s="2" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="17" t="inlineStr">
+      <c r="A6" s="3" t="inlineStr">
         <is>
           <t>Target System</t>
         </is>
       </c>
-      <c r="B6" s="18" t="inlineStr">
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <t>Supabase PostgreSQL REST API</t>
         </is>
       </c>
+      <c r="C6" s="2" t="n"/>
+      <c r="D6" s="2" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="15" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>Base URL</t>
         </is>
       </c>
-      <c r="B7" s="16" t="inlineStr">
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>https://atafeyidjdzedbktzivx.supabase.co/rest/v1</t>
         </is>
       </c>
+      <c r="C7" s="2" t="n"/>
+      <c r="D7" s="2" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="17" t="inlineStr">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>Auth Method</t>
         </is>
       </c>
-      <c r="B8" s="18" t="inlineStr">
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <t>API Key (anon/publishable)</t>
         </is>
       </c>
+      <c r="C8" s="2" t="n"/>
+      <c r="D8" s="2" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="15" t="inlineStr">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t>Virtual Users (Peak)</t>
         </is>
       </c>
-      <c r="B9" s="16" t="inlineStr">
+      <c r="B9" s="4" t="inlineStr">
         <is>
           <t>100</t>
         </is>
       </c>
+      <c r="C9" s="2" t="n"/>
+      <c r="D9" s="2" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="17" t="inlineStr">
+      <c r="A10" s="3" t="inlineStr">
         <is>
           <t>Ramp-Up Phase</t>
         </is>
       </c>
-      <c r="B10" s="18" t="inlineStr">
+      <c r="B10" s="4" t="inlineStr">
         <is>
           <t>0 → 50 VUs over 10 seconds</t>
         </is>
       </c>
+      <c r="C10" s="2" t="n"/>
+      <c r="D10" s="2" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="15" t="inlineStr">
+      <c r="A11" s="3" t="inlineStr">
         <is>
           <t>Steady State Phase</t>
         </is>
       </c>
-      <c r="B11" s="16" t="inlineStr">
+      <c r="B11" s="4" t="inlineStr">
         <is>
           <t>50 → 100 VUs over 40 seconds</t>
         </is>
       </c>
+      <c r="C11" s="2" t="n"/>
+      <c r="D11" s="2" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="17" t="inlineStr">
+      <c r="A12" s="3" t="inlineStr">
         <is>
           <t>Ramp-Down Phase</t>
         </is>
       </c>
-      <c r="B12" s="18" t="inlineStr">
+      <c r="B12" s="4" t="inlineStr">
         <is>
           <t>100 → 0 VUs over 10 seconds</t>
         </is>
       </c>
+      <c r="C12" s="2" t="n"/>
+      <c r="D12" s="2" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="15" t="inlineStr">
+      <c r="A13" s="3" t="inlineStr">
         <is>
           <t>Total Duration</t>
         </is>
       </c>
-      <c r="B13" s="16" t="inlineStr">
+      <c r="B13" s="4" t="inlineStr">
         <is>
           <t>60 seconds</t>
         </is>
       </c>
+      <c r="C13" s="2" t="n"/>
+      <c r="D13" s="2" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="17" t="inlineStr">
+      <c r="A14" s="3" t="inlineStr">
         <is>
           <t>Endpoints Tested</t>
         </is>
       </c>
-      <c r="B14" s="18" t="inlineStr">
+      <c r="B14" s="4" t="inlineStr">
         <is>
           <t>10 REST API endpoints</t>
         </is>
       </c>
+      <c r="C14" s="2" t="n"/>
+      <c r="D14" s="2" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="15" t="inlineStr">
+      <c r="A15" s="3" t="inlineStr">
         <is>
           <t>Tables Covered</t>
         </is>
       </c>
-      <c r="B15" s="16" t="inlineStr">
+      <c r="B15" s="4" t="inlineStr">
         <is>
           <t>vehicles, bookings, users, reviews, payments, notifications</t>
         </is>
       </c>
+      <c r="C15" s="2" t="n"/>
+      <c r="D15" s="2" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="17" t="inlineStr">
+      <c r="A16" s="3" t="inlineStr">
         <is>
           <t>Threshold: p(95) Duration</t>
         </is>
       </c>
-      <c r="B16" s="18" t="inlineStr">
+      <c r="B16" s="4" t="inlineStr">
         <is>
           <t>&lt; 2000 ms</t>
         </is>
       </c>
+      <c r="C16" s="2" t="n"/>
+      <c r="D16" s="2" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="15" t="inlineStr">
+      <c r="A17" s="3" t="inlineStr">
         <is>
           <t>Threshold: Error Rate</t>
         </is>
       </c>
-      <c r="B17" s="16" t="inlineStr">
+      <c r="B17" s="4" t="inlineStr">
         <is>
           <t>&lt; 10%</t>
         </is>
       </c>
+      <c r="C17" s="2" t="n"/>
+      <c r="D17" s="2" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="17" t="inlineStr">
+      <c r="A18" s="3" t="inlineStr">
         <is>
           <t>Sleep Between Iterations</t>
         </is>
       </c>
-      <c r="B18" s="18" t="inlineStr">
+      <c r="B18" s="4" t="inlineStr">
         <is>
           <t>0.5 seconds</t>
         </is>
       </c>
+      <c r="C18" s="2" t="n"/>
+      <c r="D18" s="2" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="n"/>
+      <c r="B19" s="2" t="n"/>
+      <c r="C19" s="2" t="n"/>
+      <c r="D19" s="2" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="n"/>
+      <c r="B20" s="2" t="n"/>
+      <c r="C20" s="2" t="n"/>
+      <c r="D20" s="2" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="n"/>
+      <c r="B21" s="2" t="n"/>
+      <c r="C21" s="2" t="n"/>
+      <c r="D21" s="2" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="n"/>
+      <c r="B22" s="2" t="n"/>
+      <c r="C22" s="2" t="n"/>
+      <c r="D22" s="2" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="n"/>
+      <c r="B23" s="2" t="n"/>
+      <c r="C23" s="2" t="n"/>
+      <c r="D23" s="2" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="n"/>
+      <c r="B24" s="2" t="n"/>
+      <c r="C24" s="2" t="n"/>
+      <c r="D24" s="2" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="n"/>
+      <c r="B25" s="2" t="n"/>
+      <c r="C25" s="2" t="n"/>
+      <c r="D25" s="2" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>